<commit_message>
PCO-001 Texcan MV cable: AP Package B paper, pass-through candidate to eStruxture
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019MSpbxUgW95zdfzsyfgzLv
</commit_message>
<xml_diff>
--- a/CAL3_PCO_Register_2026-10-20.xlsx
+++ b/CAL3_PCO_Register_2026-10-20.xlsx
@@ -527,7 +527,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>eStruxture direct account</t>
+          <t>AP Package B site work (PO6246)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Future-phase stock, not Phase 1 Package B scope. Prysmian stock lengths 178/187/189/197 m, 2 wk delivery, +/-5% tolerance, price subject to tariff at shipment.</t>
+          <t>AP paper: eStruxture has no account or PO with Texcan (John, 2026-10-20). Pass-through candidate AP to eStruxture: material supply only, no site work. Future-phase stock, not Phase 1 scope. Prysmian stock lengths 178/187/189/197 m, 2 wk delivery, +/-5% tolerance, price subject to tariff at shipment.</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -4126,27 +4126,27 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>eStruxture direct account</t>
+          <t>AP Package B site work (PO6246)</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>300291.44</v>
+        <v>564172.5699999999</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>AP Package B site work (PO6246)</t>
+          <t>eStruxture direct account</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>405381.13</v>
+        <v>141500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Apply rule: eStruxture direct only for active eStruxture traders; move PCO-002 and PCO-013 to AP paper
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019MSpbxUgW95zdfzsyfgzLv
</commit_message>
<xml_diff>
--- a/CAL3_PCO_Register_2026-10-20.xlsx
+++ b/CAL3_PCO_Register_2026-10-20.xlsx
@@ -592,7 +592,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>eStruxture direct account</t>
+          <t>AP Package B site work (PO6246)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -640,7 +640,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Devon told Keith to proceed 2026-10-13. Nishi re-requested approval 2026-10-20 under TP-DHC-01I. PO not yet issued. Phase 2 scope: confirm whether this is a Package B change or owner-direct.</t>
+          <t>AP paper: Magna is not an active eStruxture trader on record. Pass-through candidate AP to eStruxture as Phase 2 scope. Devon told Keith to proceed 2026-10-13. Nishi re-requested approval 2026-10-20 under TP-DHC-01I. PO not yet issued.</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>eStruxture direct account</t>
+          <t>AP Package B site work (PO6246)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>OFCI vendor scope change. Who pays camlock premium and cover freight is open. CAL3-SCS26 numbers look like owner POs: confirm contract.</t>
+          <t>AP paper: SCS is not an active eStruxture trader on record. OFCI vendor scope change; who pays camlock premium and cover freight is open. Pass-through candidate only if John directs.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -4083,7 +4083,7 @@
       <c r="C4" s="3" t="n"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Owner-direct purchases (future phase stock, OFCI vendor changes)</t>
+          <t>RULE (John, 2026-10-20): assign to eStruxture direct only where the vendor is an active trader with eStruxture, or John says so. Otherwise AP paper with pass-through flag.</t>
         </is>
       </c>
     </row>
@@ -4098,7 +4098,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4130,23 +4130,10 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>564172.5699999999</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>eStruxture direct account</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>141500</v>
+        <v>705672.5699999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add eStruxture active vendor sheet; bucket EWCL/Bolt/Uline lot rows to eStruxture direct
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019MSpbxUgW95zdfzsyfgzLv
</commit_message>
<xml_diff>
--- a/CAL3_PCO_Register_2026-10-20.xlsx
+++ b/CAL3_PCO_Register_2026-10-20.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCO Register" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lot materials (Pkg B)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contracts" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Totals" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="eStruxture vendors" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contracts" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Totals" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -900,7 +901,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Freight renegotiated (Nishi: cannot pay over $16k freight). UPS testing.</t>
+          <t>Freight renegotiated (Nishi: cannot pay over $16k freight). UPS testing. NOTE: Sunbelt is an active eStruxture direct vendor (statement 7124887, Kylie approves) but this PO is AP paper; eligible to move to eStruxture direct if John says so.</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -965,7 +966,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Second PO for 2 additional units not yet seen in folder.</t>
+          <t>Second PO for 2 additional units not yet seen in folder. NOTE: Sunbelt is an active eStruxture direct vendor; this reservation is on AP PO 2791. Eligible to move to eStruxture direct if John says so.</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1755,7 +1756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1765,6 +1766,7 @@
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1803,6 +1805,11 @@
           <t>Amount</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Contract charged</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1840,6 +1847,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1877,6 +1889,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1914,6 +1931,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1951,6 +1973,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1988,6 +2015,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2025,6 +2057,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2062,6 +2099,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2099,6 +2141,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2136,6 +2183,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2173,6 +2225,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2210,6 +2267,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2247,6 +2309,11 @@
           <t>n/a</t>
         </is>
       </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2284,6 +2351,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2321,6 +2393,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2358,6 +2435,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2395,6 +2477,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2432,6 +2519,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2469,6 +2561,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2506,6 +2603,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2543,6 +2645,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2580,6 +2687,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2617,6 +2729,11 @@
           <t>n/a</t>
         </is>
       </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2654,6 +2771,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2691,6 +2813,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2728,6 +2855,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2765,6 +2897,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2802,6 +2939,11 @@
           <t>n/a</t>
         </is>
       </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2839,6 +2981,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2876,6 +3023,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2913,6 +3065,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2950,6 +3107,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2987,6 +3149,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3024,6 +3191,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3061,6 +3233,11 @@
           <t>n/a</t>
         </is>
       </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3098,6 +3275,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3135,6 +3317,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3172,6 +3359,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3209,6 +3401,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3246,6 +3443,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3283,6 +3485,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3320,6 +3527,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3357,6 +3569,11 @@
           <t>n/a</t>
         </is>
       </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3394,6 +3611,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3431,6 +3653,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3468,6 +3695,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3505,6 +3737,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3542,6 +3779,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3579,6 +3821,11 @@
           <t>n/a</t>
         </is>
       </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3616,6 +3863,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3653,6 +3905,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3690,6 +3947,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3727,6 +3989,11 @@
           <t>in bid PDF</t>
         </is>
       </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3764,6 +4031,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3801,6 +4073,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3838,6 +4115,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3875,6 +4157,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3912,6 +4199,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3949,6 +4241,11 @@
           <t>in quote PDF</t>
         </is>
       </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3984,6 +4281,11 @@
       <c r="G60" s="2" t="inlineStr">
         <is>
           <t>n/a</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
         </is>
       </c>
     </row>
@@ -3993,6 +4295,451 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>eStruxture PO / account</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence (email, date)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Scope at CAL3</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Touches this register?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Electrical Wholesalers Calgary (EWCL)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture account; weekly statements</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>construction.finance@estruxture.com weekly statement EW20260914TO20260920, $186,536.52 of $2,672,221.04 total, approved by Kylie</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Electrical materials (lot bids S18xxxxx)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Yes: all EWCL lot rows moved to eStruxture direct</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>The Bolt Supply House</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Account 76284, NO PO, activity code CAL3 Equipment</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>construction.finance statement, Kylie approves</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Hardware / non-electrical consumables</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Yes: Bolt Supply lot row 9482309-00 moved to eStruxture direct</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Sunbelt Rentals of Canada</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture account; statement 7124887</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>construction.finance statement, Kylie approves</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Rentals (load banks, temp cooling)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Partly: PCO-006/007 are on AP POs; eligible to move if John says so</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Uline</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture account with credit limit / prepayments</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>construction.finance thread</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Consumables</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Yes: Uline lot row moved to eStruxture direct</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Binns Canada</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>PO6588</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture PO</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Collicutt Energy</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>PO4771; PO7907 ($104,450 COs)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture PO emails</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Generators</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Kolostat</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>PO7591 (Coreweave); piping POs; Master Mechanical PR00003132</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture PO emails</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>ASM Modular</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>PO7183</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>approval request email</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Modular</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Englobe</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>PO6225</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>approval request email</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Testing / inspection</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Tomecek Roney (TRL)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture consultant agreement</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>approval request email</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Structural</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>WZMH</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture consultant agreement</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>construction.finance thread</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Johnson Controls (JCI)</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>PO7762</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture PO email</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Controls</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Leeswood Construction</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Progress applications</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>construction.finance thread</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Bosch / Paladin / Rhinotek / DND / Smardt / Anjinnov / RJC / Pearl DCS</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>various eStruxture POs / rent</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>construction.finance threads</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Security, chillers, consultants, warehouse</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>NOT eStruxture direct (no account/PO found)</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr"/>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>John 2026-10-20: Texcan is AP paper (pass-through possible). No eStruxture account found for Magna, Trinity, JM Test, Crystal, Rodeo, Phoenix, Unitray, SCS, Anixter, Noramco, Gescan, Graybar, EECOL, City Electric, EBH, Alberta Breaker.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Stay on AP Package B unless John says otherwise</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4092,13 +4839,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4136,6 +4883,46 @@
         <v>705672.5699999999</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Lot material rows (amounts in bid PDFs, not extracted)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>eStruxture direct account</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="C5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>AP Package B site work (PO6246)</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="C6" s="3" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add live ACC locations export and ACC location column to PCO register
Pull the CAL-3 Locations tree (486 nodes) by API, map tender-package lot
codes to ACC block nodes in both register sheets, regenerate the xlsx.
Monday REF steps dropped per John.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CAL3_PCO_Register_2026-10-20.xlsx
+++ b/CAL3_PCO_Register_2026-10-20.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M20"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -445,12 +445,13 @@
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="50" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -491,30 +492,35 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>ACC location</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Scope</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Amount CAD (pre-tax)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Amount basis</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Kylie approval</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Status / open issue</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Source email (date)</t>
         </is>
@@ -558,28 +564,33 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
+          <t>n/a: general stock, not a location</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
           <t>751 m MV105 1C-750 35kV Cu EPR cable. Trevor: general stock, to be pulled for DHA/DHE in new year. Factory price adjustment to $211.44/m.</t>
         </is>
       </c>
-      <c r="I2" s="3" t="n">
+      <c r="J2" s="3" t="n">
         <v>158791.44</v>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>AP PO 2766 rev + Texcan OA 1750503 (tax 7,939.57 extra)</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Original approved 2026-10-05; revised PO awaiting Kylie</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>AP paper: eStruxture has no account or PO with Texcan (John, 2026-10-20). Pass-through candidate AP to eStruxture: material supply only, no site work. Future-phase stock, not Phase 1 scope. Prysmian stock lengths 178/187/189/197 m, 2 wk delivery, +/-5% tolerance, price subject to tariff at shipment.</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
@@ -623,28 +634,33 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7); DHD (CACAL3DHD, a36e5a49-739c-4f49-9f89-246a4f8fb823)</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
           <t>CAL-3 Phase 2 DHD MV terminations &amp; testing, lump sum. Same scope as DHC. OEM lead times do not meet schedule; alternates offered.</t>
         </is>
       </c>
-      <c r="I3" s="3" t="n">
+      <c r="J3" s="3" t="n">
         <v>119500</v>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Magna Q-188471 lump sum, excl. tax; extras at $135/hr blended</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Conditional (Kylie 2026-10-13): lead-time alternates must be confirmed</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>AP paper: Magna is not an active eStruxture trader on record. Pass-through candidate AP to eStruxture as Phase 2 scope. Devon told Keith to proceed 2026-10-13. Nishi re-requested approval 2026-10-20 under TP-DHC-01I. PO not yet issued.</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>2026-10-13 / 2026-10-20</t>
         </is>
@@ -688,28 +704,33 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
+          <t>CAM (CACAL3CAM, cece5fbe-b772-458c-9acd-697c84cd59d7)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
           <t>CAL-3 temp power MV terminations &amp; testing (June 2026 work). Original quote, PO issued 2026-10-20 after work done.</t>
         </is>
       </c>
-      <c r="I4" s="3" t="n">
+      <c r="J4" s="3" t="n">
         <v>18950</v>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>AP PO 2924 (matches Q-176183 total)</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Trevor approved quote 2026-06-13; PO issued 2026-10-20</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>Work done June 2026 without PO. Temp power responsibility (AP vs owner) to confirm.</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
@@ -753,28 +774,33 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
+          <t>CAM (CACAL3CAM, cece5fbe-b772-458c-9acd-697c84cd59d7)</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
           <t>Change order: 126 hrs additional labour/OT/DT ($17,010) + material ($3,122.34) for temp power setup. Cable type change, delays, extra Vista switch parts and termination kits.</t>
         </is>
       </c>
-      <c r="I5" s="3" t="n">
+      <c r="J5" s="3" t="n">
         <v>20132.34</v>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>Magna CO #001 dated 2026-09-01</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>Not approved. Keith asked 2026-10-20 whether CO can be invoiced</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>PO 2924 covers $18,950 only. CO not on PO. Decision needed: approve/reject CO and who carries it.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
@@ -818,28 +844,33 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
+          <t>not mapped: no block in lot code</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
           <t>Rental 6 x Avtron 720 kW liquid-cooled load banks + 3000A 600V dist, 6 x 800A breakers, cam cables, SPE-1000 cert, delivery and return freight. 28-day rental, Oct requirement. Nov order (7 units) separate RA.</t>
         </is>
       </c>
-      <c r="I6" s="3" t="n">
+      <c r="J6" s="3" t="n">
         <v>172310</v>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>AP PO 2812 total</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Signed by Joey/Angelo 2026-10-14; Kylie approval requested 2026-10-15; PO sent 2026-10-15</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>Kolostat (Adrien) confirms it is AP's PO. Kylie: needs a work package number so AP can invoice it. Nov RA 105267 not on this PO. Freight 14,319 + 12,519 return.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
@@ -883,28 +914,33 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
           <t>Rental 1 x 1250 kW 480 V resistive load bank + 48 x 50 ft cam cables + 16 pigtails, 4-week rate, 3rd-party freight delivery and return.</t>
         </is>
       </c>
-      <c r="I7" s="3" t="n">
+      <c r="J7" s="3" t="n">
         <v>15729</v>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>AP PO 2866 total</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Approved; PO sent 2026-10-16</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Freight renegotiated (Nishi: cannot pay over $16k freight). UPS testing. NOTE: Sunbelt is an active eStruxture direct vendor (statement 7124887, Kylie approves) but this PO is AP paper; eligible to move to eStruxture direct if John says so.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
@@ -948,28 +984,33 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
+          <t>not mapped: no block in lot code</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
           <t>Temp cooling: 2 x 5T portable AC, 400A cam distro, fan, duct, spider box cables, E&amp;D labour, 4 weeks (Oct 14 to Nov 11). Two additional 5T units requested 2026-10-13 on new PO.</t>
         </is>
       </c>
-      <c r="I8" s="3" t="n">
+      <c r="J8" s="3" t="n">
         <v>9687.549999999999</v>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Sunbelt reservation 80519077 subtotal (GST 484.39 extra)</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-15</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>Second PO for 2 additional units not yet seen in folder. NOTE: Sunbelt is an active eStruxture direct vendor; this reservation is on AP PO 2791. Eligible to move to eStruxture direct if John says so.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
@@ -1013,28 +1054,33 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
           <t>Rental Fluke 1777 power quality analyzer + 3 x 6000A flex CTs, 28-day rate Oct 19 to Nov 15. Marty expects 3 months.</t>
         </is>
       </c>
-      <c r="I9" s="3" t="n">
+      <c r="J9" s="3" t="n">
         <v>2295</v>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>AP PO 2915 / RQ24624 (28 days only)</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>Approved; PO sent 2026-10-19</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>JM Test wants credit card; Nishi asking for account terms. 3-month need = ~3x this amount.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
@@ -1078,28 +1124,33 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
+          <t>not mapped: no block in lot code</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
           <t>Equipment moves Sept 28 to Oct 2: switchgear hoist to level 2 by zoom boom, generator jack/level, exhaust piping removal, switchgear unload at warehouse. Sterling+operator, supervisor, labourers, zoom boom rental.</t>
         </is>
       </c>
-      <c r="I10" s="3" t="n">
+      <c r="J10" s="3" t="n">
         <v>29100</v>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Invoice 9812 subtotal (GST 1,455 extra); PO 2885 matches</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>Approved by Kylie 2026-10-15; PO sent 2026-10-16</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>OFCI equipment handling. Candidate for DA2 OFCI coordination line if owner agrees; otherwise Package B.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
@@ -1143,28 +1194,33 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
+          <t>not mapped: no block in lot code</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
           <t>Scanning, coring, handsawing Sept 7 to Oct 3 (electrical rooms, precast walls, exterior holes, lobby slab).</t>
         </is>
       </c>
-      <c r="I11" s="3" t="n">
+      <c r="J11" s="3" t="n">
         <v>21852.5</v>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>Sum of 4 invoice subtotals (8,060 + 300 + 8,330 + 5,162.50); GST extra; totals incl. GST 22,945.15</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>Requested 2026-10-19; Ryan confirmed work complete</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>Four invoices with no PO. Base-building penetrations: confirm AP vs GC responsibility.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
@@ -1208,26 +1264,31 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
+          <t>not mapped: no block in lot code</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
           <t>T&amp;M labour Oct 5 to 11 with signed tickets. Edward confirmed hours match timecards (truck and 3rd-party charges not tracked by AP).</t>
         </is>
       </c>
-      <c r="I12" s="3" t="n"/>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J12" s="3" t="n"/>
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>Invoice PDF is scanned; amount not extractable here</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Requested 2026-10-15 and 2026-10-16</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>Amount to be read from invoice. T&amp;M authorization lines were blank per earlier review.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
@@ -1271,28 +1332,33 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
+          <t>CSB (CACAL3CSB, d08df136-1a9f-4a3a-a7cf-3110739dbe32)</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
           <t>Cable tray, fittings, rubber roof supports (30 x 457 mm, 20 x 244 mm), freight. Heat trace, fire alarm and exhaust fan access.</t>
         </is>
       </c>
-      <c r="I13" s="3" t="n">
+      <c r="J13" s="3" t="n">
         <v>14767.11</v>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>AP PO 2822 rev 3</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-14 (rev 3 lower than prior)</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>Shipped to warehouse.</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
@@ -1336,28 +1402,33 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
+          <t>not mapped: no block in lot code</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
           <t>Camlocks sourced via US; cost impact $22k to $25k plus shipping and tariffs (SCS). Separate: battery cabinet covers crate to Edmonton for ground-bus modification, freight liability unresolved.</t>
         </is>
       </c>
-      <c r="I14" s="3" t="n">
+      <c r="J14" s="3" t="n">
         <v>22000</v>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>SCS estimate low end ($22k to $25k), not quoted</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>No approval on record</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>AP paper: SCS is not an active eStruxture trader on record. OFCI vendor scope change; who pays camlock premium and cover freight is open. Pass-through candidate only if John directs.</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
@@ -1401,28 +1472,33 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
           <t>768 m 600 kcmil Cu RW90 + 900 m #2 Cu RW90 green. Alberta stock.</t>
         </is>
       </c>
-      <c r="I15" s="3" t="n">
+      <c r="J15" s="3" t="n">
         <v>77485.2</v>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>Anixter quote total</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-19</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>Price valid 5 days, metal escalation. Flat deck freight extra.</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
@@ -1466,28 +1542,33 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
           <t>450 m RW90 250 MCM Cu (MR asked 400 m). Calgary stock.</t>
         </is>
       </c>
-      <c r="I16" s="3" t="n">
+      <c r="J16" s="3" t="n">
         <v>16776</v>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>Texcan quote (450 m x $37.28)</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-20</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>450 vs 400 m not resolved; metal adjustment at shipment.</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
@@ -1531,24 +1612,29 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
           <t>94 m 250 MCM Cu RW90 (30 m + 64 m). Only supplier with stock.</t>
         </is>
       </c>
-      <c r="I17" s="3" t="n">
+      <c r="J17" s="3" t="n">
         <v>3815.46</v>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>Noramco quote</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-16</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
@@ -1592,28 +1678,33 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
+          <t>CSB (CACAL3CSB, d08df136-1a9f-4a3a-a7cf-3110739dbe32)</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
           <t>Wiremold floor box parts for NOC room missed box + $200 expedite freight.</t>
         </is>
       </c>
-      <c r="I18" s="3" t="n">
+      <c r="J18" s="3" t="n">
         <v>1153.05</v>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>Gescan quote incl. freight</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>Requested 2026-10-16</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>7 to 15 working days from Wiremold.</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
@@ -1657,24 +1748,29 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
+          <t>CSB (CACAL3CSB, d08df136-1a9f-4a3a-a7cf-3110739dbe32)</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
           <t>15 x 4 in square covers (30 requested, 15 in stock).</t>
         </is>
       </c>
-      <c r="I19" s="3" t="n">
+      <c r="J19" s="3" t="n">
         <v>459.92</v>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>Gescan quote (30 pcs); 15 pcs = 229.96</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>Requested 2026-10-16</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
@@ -1718,28 +1814,33 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
           <t>150 x T&amp;B universal clamps (tray down), air freight from Quebec. 350 requested.</t>
         </is>
       </c>
-      <c r="I20" s="3" t="n">
+      <c r="J20" s="3" t="n">
         <v>868</v>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>Graybar quote: 828 + 40 freight (GST 43.40 extra)</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-20</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>Remaining 200 to be sourced elsewhere.</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
@@ -1756,17 +1857,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1787,25 +1889,30 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>ACC location</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Note from thread</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Kylie approval</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Contract charged</t>
         </is>
@@ -1829,25 +1936,30 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>n/a: no lot code</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>Jeff Bosch chasing approval</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -1871,25 +1983,30 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
           <t>wire, 2 to 3 day ETA</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -1913,25 +2030,30 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>CSB (CACAL3CSB, d08df136-1a9f-4a3a-a7cf-3110739dbe32)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
           <t>in-stock items only</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -1955,25 +2077,30 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t>CSB (CACAL3CSB, d08df136-1a9f-4a3a-a7cf-3110739dbe32)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
           <t>in-stock items only</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -1997,25 +2124,30 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
           <t>stocked, pickup same day</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -2039,25 +2171,30 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
+          <t>CAM (CACAL3CAM, cece5fbe-b772-458c-9acd-697c84cd59d7)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
           <t>spider box, in stock</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -2081,25 +2218,30 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
+          <t>CSB (CACAL3CSB, d08df136-1a9f-4a3a-a7cf-3110739dbe32); DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
           <t>all in stock; acknowledged, ships Monday</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-15</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -2123,25 +2265,30 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
+          <t>n/a: general stock, not a location</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t>in stock + under 1 week; MR revised</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Requested 2026-10-16</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -2165,25 +2312,30 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
+          <t>CAM (CACAL3CAM, cece5fbe-b772-458c-9acd-697c84cd59d7)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
           <t>in-stock only; HAL UHBS2 substituted for RENO HBU</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Requested 2026-10-16</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -2207,25 +2359,30 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
           <t>stocked</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-16</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -2249,25 +2406,30 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
           <t>1 item in stock</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-16</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -2291,25 +2453,30 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
           <t>rubber edge, short 2000; 30 pcs 50 ft</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Requested 2026-10-16</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -2333,25 +2500,30 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
+          <t>CSB (CACAL3CSB, d08df136-1a9f-4a3a-a7cf-3110739dbe32)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
           <t>all in stock</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-15</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -2375,25 +2547,30 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
           <t>in stock</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-15</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -2417,25 +2594,30 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
           <t>in stock</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-15</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -2459,25 +2641,30 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
+          <t>CSB (CACAL3CSB, d08df136-1a9f-4a3a-a7cf-3110739dbe32)</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
           <t>all in stock</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-15</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -2501,25 +2688,30 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
           <t>3 items</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-15</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -2543,25 +2735,30 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
           <t>stock, weekend work</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-15</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -2585,25 +2782,30 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
           <t>all non-electrical items</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-15 (after call)</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -2627,25 +2829,30 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
           <t>in-stock items; 2 not stocked</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -2669,25 +2876,30 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
+          <t>CSB (CACAL3CSB, d08df136-1a9f-4a3a-a7cf-3110739dbe32)</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
           <t>4 week ETA</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -2711,25 +2923,30 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
+          <t>CSB (CACAL3CSB, d08df136-1a9f-4a3a-a7cf-3110739dbe32)</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
           <t>PVC boxes declined</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>Declined</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -2753,25 +2970,30 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
           <t>in stock</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -2795,25 +3017,30 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
+          <t>DHD (CACAL3DHD, a36e5a49-739c-4f49-9f89-246a4f8fb823)</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
           <t>multiple options</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="I25" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -2837,25 +3064,30 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
+          <t>CSB (CACAL3CSB, d08df136-1a9f-4a3a-a7cf-3110739dbe32)</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
           <t>blue liquid tight; pre-approved by Angelo</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-15</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -2879,25 +3111,30 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
+          <t>CSB (CACAL3CSB, d08df136-1a9f-4a3a-a7cf-3110739dbe32)</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
           <t>basket tray covers, only supplier before month end</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>Requested 2026-10-14</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -2921,25 +3158,30 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
+          <t>CSB (CACAL3CSB, d08df136-1a9f-4a3a-a7cf-3110739dbe32)</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
           <t>Brady lockbox LOTO</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-14</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -2963,25 +3205,30 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
           <t>in stock; ships Friday</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-14</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -3005,25 +3252,30 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
           <t>30 m in stock</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-14</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -3047,25 +3299,30 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
           <t>2 items</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-14</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -3089,25 +3346,30 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
           <t>all in stock</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-14</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -3131,25 +3393,30 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
+          <t>CSB (CACAL3CSB, d08df136-1a9f-4a3a-a7cf-3110739dbe32)</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
           <t>in-stock items; 10 KO fillers sold out</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-14</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -3173,25 +3440,30 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
           <t>1 week ETA items only</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -3215,25 +3487,30 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
           <t>slotted shipped in error; RMA, solid in stock</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>n/a (RMA)</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -3257,25 +3534,30 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
+          <t>DHD (CACAL3DHD, a36e5a49-739c-4f49-9f89-246a4f8fb823)</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
           <t>4 options</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="I36" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -3299,25 +3581,30 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
+          <t>n/a: no lot code</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
           <t>motion sensor switch (Devon)</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-14</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="I37" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -3341,25 +3628,30 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
           <t>18 in stock + 100 air freight</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-14</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="I38" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -3383,25 +3675,30 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
           <t>in-stock items</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-14</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G39" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H39" s="2" t="inlineStr">
+      <c r="I39" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -3425,25 +3722,30 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
           <t>20 pcs in stock</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-14</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="I40" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -3467,25 +3769,30 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
+          <t>DHD (CACAL3DHD, a36e5a49-739c-4f49-9f89-246a4f8fb823)</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
           <t>in-stock items</t>
         </is>
       </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-14</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G41" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H41" s="2" t="inlineStr">
+      <c r="I41" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -3509,25 +3816,30 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
+          <t>CSB (CACAL3CSB, d08df136-1a9f-4a3a-a7cf-3110739dbe32)</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
           <t>in-stock items</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-14</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="I42" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -3551,25 +3863,30 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
           <t>rubber edge, $60/roll vs EECOL $500/roll</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="F43" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-14</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="G43" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G43" s="2" t="inlineStr">
+      <c r="H43" s="2" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="I43" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -3593,25 +3910,30 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
+          <t>CSB (CACAL3CSB, d08df136-1a9f-4a3a-a7cf-3110739dbe32)</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
           <t>extra exit signs, Joey pre-approved</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-14</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -3635,25 +3957,30 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
           <t>all items incl. short lead</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="F45" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-14</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="G45" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G45" s="2" t="inlineStr">
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H45" s="2" t="inlineStr">
+      <c r="I45" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -3677,25 +4004,30 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
           <t>in stock + MR qty 20 line 2</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-14</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="I46" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -3719,25 +4051,30 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
           <t>in-stock items</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-14</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G47" s="2" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="I47" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -3761,25 +4098,30 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
+          <t>CAM (CACAL3CAM, cece5fbe-b772-458c-9acd-697c84cd59d7)</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
           <t>all in stock</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-14</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr">
+      <c r="I48" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -3803,25 +4145,30 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
+          <t>CSB (CACAL3CSB, d08df136-1a9f-4a3a-a7cf-3110739dbe32)</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
           <t>only stocked at Uline</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>Requested 2026-10-14</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr">
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="G49" s="2" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H49" s="2" t="inlineStr">
+      <c r="I49" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -3845,25 +4192,30 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
+          <t>CSB (CACAL3CSB, d08df136-1a9f-4a3a-a7cf-3110739dbe32)</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
           <t>2 items</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-13</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr">
+      <c r="I50" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -3887,25 +4239,30 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
           <t>4 items in stock</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="F51" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-13</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
+      <c r="G51" s="2" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="G51" s="2" t="inlineStr">
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H51" s="2" t="inlineStr">
+      <c r="I51" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -3929,25 +4286,30 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
           <t>60 m or 45 m options, 2 to 6 wk</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr">
+      <c r="I52" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -3971,25 +4333,30 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
+          <t>CSB (CACAL3CSB, d08df136-1a9f-4a3a-a7cf-3110739dbe32)</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
           <t>3 options</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="F53" s="2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
+      <c r="G53" s="2" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="G53" s="2" t="inlineStr">
+      <c r="H53" s="2" t="inlineStr">
         <is>
           <t>in bid PDF</t>
         </is>
       </c>
-      <c r="H53" s="2" t="inlineStr">
+      <c r="I53" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -4013,25 +4380,30 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
+          <t>n/a: general stock, not a location</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
           <t>bulk order, Allan; PO done, OA received, no ETA</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>Approved (prior)</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr">
+      <c r="H54" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H54" s="2" t="inlineStr">
+      <c r="I54" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -4055,25 +4427,30 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
           <t>rubber edge; Kylie flagged $500/roll vs Amazon $60</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="F55" s="2" t="inlineStr">
         <is>
           <t>Challenged</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
+      <c r="G55" s="2" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="G55" s="2" t="inlineStr">
+      <c r="H55" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H55" s="2" t="inlineStr">
+      <c r="I55" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -4097,25 +4474,30 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
           <t>1 item</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-13</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="G56" s="2" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr">
+      <c r="I56" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -4139,25 +4521,30 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
+          <t>CSB (CACAL3CSB, d08df136-1a9f-4a3a-a7cf-3110739dbe32)</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
           <t>in stock</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="F57" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-13</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
+      <c r="G57" s="2" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="G57" s="2" t="inlineStr">
+      <c r="H57" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H57" s="2" t="inlineStr">
+      <c r="I57" s="2" t="inlineStr">
         <is>
           <t>eStruxture direct account</t>
         </is>
@@ -4181,25 +4568,30 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
           <t>see Kylie note</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-13</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="G58" s="2" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="H58" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr">
+      <c r="I58" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -4223,25 +4615,30 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
+          <t>DHC (CACAL3DHC, 8e694ee8-5818-4a4a-8ff1-06c1ed0c51a7)</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
           <t>14 x #6 lugs</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="F59" s="2" t="inlineStr">
         <is>
           <t>Approved 2026-10-06</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr">
+      <c r="G59" s="2" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="G59" s="2" t="inlineStr">
+      <c r="H59" s="2" t="inlineStr">
         <is>
           <t>in quote PDF</t>
         </is>
       </c>
-      <c r="H59" s="2" t="inlineStr">
+      <c r="I59" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>
@@ -4265,25 +4662,30 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
+          <t>n/a: no lot code</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
           <t>LLSCO lug shortage, 22+ wk leads; air freight option</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="F60" s="2" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="G60" s="2" t="inlineStr">
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H60" s="2" t="inlineStr">
+      <c r="I60" s="2" t="inlineStr">
         <is>
           <t>AP Package B site work (PO6246)</t>
         </is>

</xml_diff>